<commit_message>
Fix: move _run_pipeline above entry point, remove dead main()
- The NameError (line 408) was caused by _run_pipeline being defined
  *after* the if __name__ block that calls it. Moved the definition above
  the entry point and removed the duplicate at the bottom.
- Removed the now-dead old main() (the entry point now routes through
  _run_pipeline).
- Safe-destroy guard for winfo_exists already in place.
</commit_message>
<xml_diff>
--- a/4 Application monitoring/Application_Tracker.xlsx
+++ b/4 Application monitoring/Application_Tracker.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -499,6 +499,195 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CV-20260912-0001</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Job Description (text)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>(pasted text)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260912-0001.txt</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>JD collected — awaiting document generation</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Manifest: 4 Application monitoring\manifests\CV-20260912-0001.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CV-20260912-0002</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Job Description (text)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>(pasted text)</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260912-0002.txt</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>JD collected — awaiting document generation</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Manifest: 4 Application monitoring\manifests\CV-20260912-0002.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CV-20260912-0003</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Job Description (text)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(pasted text)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260912-0003.txt</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>JD collected — awaiting document generation</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Manifest: 4 Application monitoring\manifests\CV-20260912-0003.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CV-20260912-0004</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Job Description (file)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(pasted text)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260912-0004.txt</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>JD collected — awaiting document generation</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Manifest: 4 Application monitoring\manifests\CV-20260912-0004.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CV-20260912-0005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Job Description (file)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(pasted text)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260912-0005.txt</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>JD collected — awaiting document generation</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Manifest: 4 Application monitoring\manifests\CV-20260912-0005.txt</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Generate artifacts for serial CV-20260912-0005 + update tracker
- Match & Gap Analysis -> 2 Job description/CV-20260912-0005_MATCH_GAP.txt
- 3 tailored CVs -> 3 Custom CV/CV-20260912-0005_CV{1,2,3}.txt
- 5 cover letters -> 5 Custom Cover Letter/CV-20260912-0005_CL{1..5}.txt
- 6 interview-prep STAR answers -> 6 Interview Prep/CV-20260912-0005_IP{1..6}.txt
- Excel tracker row updated: Status='Documents generated (15)', Documents Generated lists all 15 paths
- Content derived strictly from base CV (1 Source/SONG Ernest - CV v1.typ); no invented metrics
</commit_message>
<xml_diff>
--- a/4 Application monitoring/Application_Tracker.xlsx
+++ b/4 Application monitoring/Application_Tracker.xlsx
@@ -653,9 +653,6 @@
           <t>CV-20260912-0005</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>2026-09-12</t>
@@ -678,10 +675,14 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>JD collected — awaiting document generation</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
+          <t>Documents generated (15)</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260912-0005_MATCH_GAP.txt; 3 Custom CV\CV-20260912-0005_CV1.txt; 3 Custom CV\CV-20260912-0005_CV2.txt; 3 Custom CV\CV-20260912-0005_CV3.txt; 5 Custom Cover Letter\CV-20260912-0005_CL1.txt; 5 Custom Cover Letter\CV-20260912-0005_CL2.txt; 5 Custom Cover Letter\CV-20260912-0005_CL3.txt; 5 Custom Cover Letter\CV-20260912-0005_CL4.txt; 5 Custom Cover Letter\CV-20260912-0005_CL5.txt; 6 Interview Prep\CV-20260912-0005_IP1.txt; 6 Interview Prep\CV-20260912-0005_IP2.txt; 6 Interview Prep\CV-20260912-0005_IP3.txt; 6 Interview Prep\CV-20260912-0005_IP4.txt; 6 Interview Prep\CV-20260912-0005_IP5.txt; 6 Interview Prep\CV-20260912-0005_IP6.txt</t>
+        </is>
+      </c>
       <c r="K6" t="inlineStr">
         <is>
           <t>Manifest: 4 Application monitoring\manifests\CV-20260912-0005.txt</t>

</xml_diff>

<commit_message>
Fix: resolve Typst compile errors from incomplete callout string quotes
- Correct the JD-relevance profile-highlight callout in gen_cv_typ.py and _apply_gen.py:
  the #text() callout quote was unterminated ("bold)[ -> "bold")[), which caused cascading
  'unclosed delimiter' / 'expected comma' errors across the grid/body.
- Regenerate JD-tailored .typ and compile CV-20260912-0005_CV1.pdf (clean compile, no errors).
- Add pipeline helpers: _apply_body.py, _fix_qlik.py, company_profile.py, generate_documents.py.
- Update run_cv_builder.bat and PROJECT_LOG.md.
- Regenerate serial CV artifacts (CV-0006/0007, cover letter, interview prep) and prune old CV2/CV3.
</commit_message>
<xml_diff>
--- a/4 Application monitoring/Application_Tracker.xlsx
+++ b/4 Application monitoring/Application_Tracker.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -689,6 +689,85 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CV-20260912-0006</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Job Description (text)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(pasted text)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260912-0006.txt</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>JD collected — awaiting document generation</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Manifest: 4 Application monitoring\manifests\CV-20260912-0006.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CV-20260912-0007</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Job Description (text)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(pasted text)</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260912-0007.txt</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260912-0007_CL1.docx; 6 Interview Prep\CV-20260912-0007_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-13: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix gen_cv_typ: remove shadowing duplicate main(); plain run now generates CV + PDF (was only printing JD)
</commit_message>
<xml_diff>
--- a/4 Application monitoring/Application_Tracker.xlsx
+++ b/4 Application monitoring/Application_Tracker.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -768,6 +768,47 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CV-20260914-0008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Job Description (text)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(pasted text)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260914-0008.txt</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>JD collected — awaiting document generation</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Manifest: 4 Application monitoring\manifests\CV-20260914-0008.txt</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add generated artifacts (JD text, CV PDF/typ, cover letters, interview prep, manifests, tracker) to source; restore original .gitignore
</commit_message>
<xml_diff>
--- a/4 Application monitoring/Application_Tracker.xlsx
+++ b/4 Application monitoring/Application_Tracker.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1536,6 +1536,1268 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CV-20260915-0027</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0027.txt</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0027_CL1.docx; 6 Interview Prep\CV-20260915-0027_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>CV-20260915-0028</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0028.txt</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0028_CL1.docx; 6 Interview Prep\CV-20260915-0028_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>CV-20260915-0029</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0029.txt</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0029_CL1.docx; 6 Interview Prep\CV-20260915-0029_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>CV-20260915-0030</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0030.txt</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>JD collected — awaiting document generation</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Manifest: 4 Application monitoring\manifests\CV-20260915-0030.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>CV-20260915-0031</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0031.txt</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0031_CL1.docx; 6 Interview Prep\CV-20260915-0031_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>CV-20260915-0032</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0032.txt</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0032_CL1.docx; 6 Interview Prep\CV-20260915-0032_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>CV-20260915-0033</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0033.txt</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>JD collected — awaiting document generation</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Manifest: 4 Application monitoring\manifests\CV-20260915-0033.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>CV-20260915-0034</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0034.txt</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>JD collected — awaiting document generation</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Manifest: 4 Application monitoring\manifests\CV-20260915-0034.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>CV-20260915-0035</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0035.txt</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>JD collected — awaiting document generation</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Manifest: 4 Application monitoring\manifests\CV-20260915-0035.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>CV-20260915-0036</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0036.txt</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>JD collected — awaiting document generation</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Manifest: 4 Application monitoring\manifests\CV-20260915-0036.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>CV-20260915-0037</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0037.txt</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>JD collected — awaiting document generation</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Manifest: 4 Application monitoring\manifests\CV-20260915-0037.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>CV-20260915-0038</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0038.txt</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>JD collected — awaiting document generation</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Manifest: 4 Application monitoring\manifests\CV-20260915-0038.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>CV-20260915-0039</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0039.txt</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0039_CL1.docx; 6 Interview Prep\CV-20260915-0039_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>CV-20260915-0040</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0040.txt</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>JD collected — awaiting document generation</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Manifest: 4 Application monitoring\manifests\CV-20260915-0040.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>CV-20260915-0041</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0041.txt</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0041_CL1.docx; 6 Interview Prep\CV-20260915-0041_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>CV-20260915-0042</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0042.txt</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0042_CL1.docx; 6 Interview Prep\CV-20260915-0042_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>CV-20260915-0043</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0043.txt</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0043_CL1.docx; 6 Interview Prep\CV-20260915-0043_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>CV-20260915-0044</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0044.txt</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0044_CL1.docx; 6 Interview Prep\CV-20260915-0044_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>CV-20260915-0045</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0045.txt</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0045_CL1.docx; 6 Interview Prep\CV-20260915-0045_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>CV-20260915-0046</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0046.txt</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0046_CL1.docx; 6 Interview Prep\CV-20260915-0046_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>CV-20260915-0047</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0047.txt</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0047_CL1.docx; 6 Interview Prep\CV-20260915-0047_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>CV-20260915-0048</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0048.txt</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0048_CL1.docx; 6 Interview Prep\CV-20260915-0048_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>CV-20260915-0049</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0049.txt</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0049_CL1.docx; 6 Interview Prep\CV-20260915-0049_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>CV-20260915-0050</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0050.txt</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0050_CL1.docx; 6 Interview Prep\CV-20260915-0050_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>CV-20260915-0051</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0051.txt</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0051_CL1.docx; 6 Interview Prep\CV-20260915-0051_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>CV-20260915-0052</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0052.txt</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0052_CL1.docx; 6 Interview Prep\CV-20260915-0052_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>CV-20260915-0053</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0053.txt</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0053_CL1.docx; 6 Interview Prep\CV-20260915-0053_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>CV-20260915-0054</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0054.txt</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0054_CL1.docx; 6 Interview Prep\CV-20260915-0054_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>CV-20260915-0055</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0055.txt</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0055_CL1.docx; 6 Interview Prep\CV-20260915-0055_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>CV-20260915-0056</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0056.txt</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0056_CL1.docx; 6 Interview Prep\CV-20260915-0056_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>CV-20260915-0057</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0057.txt</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0057_CL1.docx; 6 Interview Prep\CV-20260915-0057_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
cv: tailor CV PDF position to the target JD (auto/CLI title) instead of hardcoding 'Finance Domain Leader'
</commit_message>
<xml_diff>
--- a/4 Application monitoring/Application_Tracker.xlsx
+++ b/4 Application monitoring/Application_Tracker.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K58"/>
+  <dimension ref="A1:K63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2798,6 +2798,216 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>CV-20260915-0058</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0058.txt</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0058_CL1.docx; 6 Interview Prep\CV-20260915-0058_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>CV-20260915-0059</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0059.txt</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0059_CL1.docx; 6 Interview Prep\CV-20260915-0059_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>CV-20260915-0060</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0060.txt</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0060_CL1.docx; 6 Interview Prep\CV-20260915-0060_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>CV-20260915-0061</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0061.txt</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0061_CL1.docx; 6 Interview Prep\CV-20260915-0061_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>CV-20260915-0062</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/pulse/lead-bi-analytics-consultant-brussels-hybrid-freelance-jeremie-meba-gsqme/</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260915-0062.txt</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>3 Custom CV\CV-20260912-0005_CV1.pdf; 5 Custom Cover Letter\CV-20260915-0062_CL1.docx; 6 Interview Prep\CV-20260915-0062_IP1.docx</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Generated 2026-09-15: CV + 1 cover letter + 1 interview prep</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
generation: add hidden debug log (.generation_debug.log) for diagnosing LLM/typst failures
</commit_message>
<xml_diff>
--- a/4 Application monitoring/Application_Tracker.xlsx
+++ b/4 Application monitoring/Application_Tracker.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -499,6 +499,85 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CV-20260916-0001</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Job Description (text)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>(pasted text)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260916-0001.txt</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>JD collected — awaiting document generation</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Manifest: 4 Application monitoring\manifests\CV-20260916-0001.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CV-20260917-0002</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Job Description (text)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>(pasted text)</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2 Job description\CV-20260917-0002.txt</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Documents generated</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>C:\MyDev\MyCV\3 Custom CV\CV-20260917-0002_CV1.pdf; C:\MyDev\MyCV\3 Custom CV\CV-20260917-0002_CV2.pdf; C:\MyDev\MyCV\3 Custom CV\CV-20260917-0002_CV3.pdf; C:\MyDev\MyCV\2 Job description\CV-20260917-0002_MATCH_GAP.txt</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Generated 20260917: 3 CV PDF(s) + 0 cover letter(s) + 0 interview prep(s)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>